<commit_message>
fixed api issue and changes some UI
</commit_message>
<xml_diff>
--- a/data/data_example.xlsx
+++ b/data/data_example.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kamrynmansfield/College/UTK/research/TRiP_app/TRiP_app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFB320E-261E-8D40-9491-4D40011BD380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D80B8D-969D-BB40-B0C7-2D55F203FDA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="660" windowWidth="19580" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$1594</definedName>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1598" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1617" uniqueCount="33">
   <si>
     <t>month</t>
   </si>
@@ -120,11 +121,17 @@
   <si>
     <t>79</t>
   </si>
+  <si>
+    <t>brt</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -150,7 +157,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -158,16 +165,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -183,6 +217,295 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>800100</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>107979</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>159395</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Right Brace 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5DF34382-5B76-F8E7-05B3-EB1C71601EE0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="5958228" y="-216951"/>
+          <a:ext cx="241659" cy="3935406"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightBrace">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>107979</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>159395</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Right Brace 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11DFD737-2FB6-53A2-14CF-B9BD8D8AF110}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="8346188" y="1343195"/>
+          <a:ext cx="241659" cy="815114"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightBrace">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>279400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>19336</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>596900</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>95536</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="TextBox 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B13DEFC-C998-B4A4-C54A-A09765DB9A61}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5246283" y="1351036"/>
+          <a:ext cx="1741751" cy="266443"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Required</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>355600</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>19336</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>444500</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>95536</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="TextBox 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8ED3F25A-5B84-3F53-47F3-5BCF31FAF218}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7574547" y="1351036"/>
+          <a:ext cx="1744528" cy="266443"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Optional</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4118,8 +4441,8 @@
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A215" t="s">
-        <v>14</v>
+      <c r="A215">
+        <v>19</v>
       </c>
       <c r="B215">
         <v>1</v>
@@ -27220,4 +27543,326 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA9F1A4E-BA4F-3F46-9A17-7FC883E35C3A}">
+  <dimension ref="F11:K27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="7" max="7" width="7.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="11" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F11" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="4">
+        <v>1</v>
+      </c>
+      <c r="H12" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I12" s="5">
+        <v>12102</v>
+      </c>
+      <c r="J12" s="5">
+        <v>10639.96</v>
+      </c>
+      <c r="K12" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="4">
+        <v>2</v>
+      </c>
+      <c r="H13" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I13" s="5">
+        <v>16966</v>
+      </c>
+      <c r="J13" s="5">
+        <v>11767.44</v>
+      </c>
+      <c r="K13" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="4">
+        <v>3</v>
+      </c>
+      <c r="H14" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I14" s="5">
+        <v>16886</v>
+      </c>
+      <c r="J14" s="5">
+        <v>11760.77</v>
+      </c>
+      <c r="K14" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F15" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="4">
+        <v>4</v>
+      </c>
+      <c r="H15" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I15" s="5">
+        <v>18486</v>
+      </c>
+      <c r="J15" s="5">
+        <v>12328.96</v>
+      </c>
+      <c r="K15" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="4">
+        <v>5</v>
+      </c>
+      <c r="H16" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I16" s="5">
+        <v>17199</v>
+      </c>
+      <c r="J16" s="5">
+        <v>12323.4</v>
+      </c>
+      <c r="K16" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F17" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="4">
+        <v>6</v>
+      </c>
+      <c r="H17" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I17" s="5">
+        <v>14051</v>
+      </c>
+      <c r="J17" s="5">
+        <v>11185.92</v>
+      </c>
+      <c r="K17" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="4">
+        <v>7</v>
+      </c>
+      <c r="H18" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I18" s="5">
+        <v>15298</v>
+      </c>
+      <c r="J18" s="5">
+        <v>11198.2</v>
+      </c>
+      <c r="K18" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F19" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="4">
+        <v>1</v>
+      </c>
+      <c r="H19" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I19" s="5">
+        <v>9365</v>
+      </c>
+      <c r="J19" s="5">
+        <v>9243.24</v>
+      </c>
+      <c r="K19" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F20" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="4">
+        <v>2</v>
+      </c>
+      <c r="H20" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I20" s="5">
+        <v>12053</v>
+      </c>
+      <c r="J20" s="5">
+        <v>10216.209999999999</v>
+      </c>
+      <c r="K20" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F21" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="4">
+        <v>3</v>
+      </c>
+      <c r="H21" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I21" s="5">
+        <v>11226</v>
+      </c>
+      <c r="J21" s="5">
+        <v>10216.209999999999</v>
+      </c>
+      <c r="K21" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F22" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="4">
+        <v>4</v>
+      </c>
+      <c r="H22" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I22" s="5">
+        <v>11725</v>
+      </c>
+      <c r="J22" s="5">
+        <v>10702.7</v>
+      </c>
+      <c r="K22" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F23" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="4">
+        <v>5</v>
+      </c>
+      <c r="H23" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I23" s="5">
+        <v>11219</v>
+      </c>
+      <c r="J23" s="5">
+        <v>10702.7</v>
+      </c>
+      <c r="K23" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F24" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="4">
+        <v>6</v>
+      </c>
+      <c r="H24" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I24" s="5">
+        <v>9413</v>
+      </c>
+      <c r="J24" s="5">
+        <v>9729.73</v>
+      </c>
+      <c r="K24" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="F25" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="4">
+        <v>7</v>
+      </c>
+      <c r="H25" s="4">
+        <v>2024</v>
+      </c>
+      <c r="I25" s="5">
+        <v>9875</v>
+      </c>
+      <c r="J25" s="5">
+        <v>9859.7900000000009</v>
+      </c>
+      <c r="K25" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="6:11" x14ac:dyDescent="0.2">
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>